<commit_message>
Update RheoBoard V9 BOM spreadsheet
Refreshes `RheoBoard_V9.xlsx` with the latest bill of materials revisions for the V9 PCB.
</commit_message>
<xml_diff>
--- a/RheoBoard-PCB_V9/Bill of Materials/RheoBoard_V9.xlsx
+++ b/RheoBoard-PCB_V9/Bill of Materials/RheoBoard_V9.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HoangVuong\RheoBoard_Adafruit_V6\RheoBoard_Adafruit_V6\MICROPROCESSOR\Project Outputs for MICROPROCESSOR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50E39766-B97D-4C3A-9B52-5274D1099DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{265CD967-4EB8-4120-8E44-AE91A19003F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{45DACFD9-4B98-4724-AE9C-7AAFE8B30869}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="171">
   <si>
     <t>Line #</t>
   </si>
@@ -73,9 +73,6 @@
   </si>
   <si>
     <t>Supplier Subtotal 1</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>100nF</t>
@@ -262,9 +259,6 @@
     <t>4.7uH</t>
   </si>
   <si>
-    <t>IND MOI 1W2T 4.7uH 20% 5A 0420 SMD</t>
-  </si>
-  <si>
     <t>L1</t>
   </si>
   <si>
@@ -554,6 +548,9 @@
   </si>
   <si>
     <t>Lite-On LED Red 1206</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 4.7uH CD74R SMD</t>
   </si>
 </sst>
 </file>
@@ -1000,13 +997,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="E2" s="1">
         <v>2</v>
@@ -1025,13 +1022,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>17</v>
       </c>
       <c r="E3" s="1">
         <v>2</v>
@@ -1050,13 +1047,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E4" s="1">
         <v>2</v>
@@ -1075,13 +1072,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="D5" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E5" s="1">
         <v>8</v>
@@ -1100,13 +1097,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>21</v>
       </c>
       <c r="E6" s="1">
         <v>5</v>
@@ -1125,13 +1122,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="D7" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E7" s="1">
         <v>1</v>
@@ -1150,13 +1147,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E8" s="1">
         <v>1</v>
@@ -1175,13 +1172,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="E9" s="1">
         <v>3</v>
@@ -1190,10 +1187,10 @@
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>28</v>
       </c>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
@@ -1204,13 +1201,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="E10" s="1">
         <v>1</v>
@@ -1219,10 +1216,10 @@
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
       <c r="I10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J10" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>28</v>
       </c>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
@@ -1233,13 +1230,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="E11" s="1">
         <v>1</v>
@@ -1248,10 +1245,10 @@
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
       <c r="I11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J11" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
@@ -1262,13 +1259,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>38</v>
       </c>
       <c r="E12" s="1">
         <v>1</v>
@@ -1287,13 +1284,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E13" s="1">
         <v>4</v>
@@ -1302,10 +1299,10 @@
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J13" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
@@ -1316,13 +1313,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="E14" s="1">
         <v>1</v>
@@ -1341,13 +1338,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="E15" s="1">
         <v>5</v>
@@ -1356,10 +1353,10 @@
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
@@ -1370,29 +1367,29 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>47</v>
       </c>
       <c r="E16" s="1">
         <v>1</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="H16" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="H16" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="I16" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
@@ -1403,31 +1400,31 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E17" s="1">
         <v>5</v>
       </c>
       <c r="F17" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="H17" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="H17" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="I17" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
@@ -1438,13 +1435,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="E18" s="1">
         <v>1</v>
@@ -1453,10 +1450,10 @@
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="J18" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
@@ -1467,13 +1464,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>60</v>
       </c>
       <c r="E19" s="1">
         <v>1</v>
@@ -1482,10 +1479,10 @@
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
@@ -1496,13 +1493,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>64</v>
       </c>
       <c r="E20" s="1">
         <v>4</v>
@@ -1521,13 +1518,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C21" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>66</v>
       </c>
       <c r="E21" s="1">
         <v>1</v>
@@ -1546,13 +1543,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="E22" s="1">
         <v>1</v>
@@ -1571,13 +1568,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="D23" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>72</v>
       </c>
       <c r="E23" s="1">
         <v>1</v>
@@ -1596,13 +1593,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>75</v>
       </c>
       <c r="E24" s="1">
         <v>1</v>
@@ -1621,13 +1618,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C25" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="E25" s="1">
         <v>1</v>
@@ -1646,13 +1643,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>79</v>
       </c>
       <c r="E26" s="1">
         <v>8</v>
@@ -1671,13 +1668,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>82</v>
       </c>
       <c r="E27" s="1">
         <v>6</v>
@@ -1686,10 +1683,10 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
@@ -1700,13 +1697,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>86</v>
       </c>
       <c r="E28" s="1">
         <v>2</v>
@@ -1715,10 +1712,10 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
@@ -1729,13 +1726,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>90</v>
       </c>
       <c r="E29" s="1">
         <v>1</v>
@@ -1754,13 +1751,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E30" s="1">
         <v>1</v>
@@ -1779,13 +1776,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E31" s="1">
         <v>1</v>
@@ -1804,13 +1801,13 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E32" s="1">
         <v>1</v>
@@ -1829,19 +1826,19 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E33" s="1">
+        <v>1</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="E33" s="1">
-        <v>1</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
@@ -1856,13 +1853,13 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E34" s="1">
         <v>1</v>
@@ -1881,13 +1878,13 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E35" s="1">
         <v>2</v>
@@ -1906,13 +1903,13 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E36" s="1">
         <v>1</v>
@@ -1931,13 +1928,13 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E37" s="1">
         <v>4</v>
@@ -1956,13 +1953,13 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E38" s="1">
         <v>1</v>
@@ -1981,13 +1978,13 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E39" s="1">
         <v>5</v>
@@ -2006,13 +2003,13 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E40" s="1">
         <v>1</v>
@@ -2031,13 +2028,13 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E41" s="1">
         <v>2</v>
@@ -2056,13 +2053,13 @@
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E42" s="1">
         <v>2</v>
@@ -2081,13 +2078,13 @@
         <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E43" s="1">
         <v>2</v>
@@ -2106,13 +2103,13 @@
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>120</v>
       </c>
       <c r="E44" s="1">
         <v>4</v>
@@ -2121,10 +2118,10 @@
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
       <c r="I44" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="K44" s="1"/>
       <c r="L44" s="1"/>
@@ -2135,13 +2132,13 @@
         <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>125</v>
       </c>
       <c r="E45" s="1">
         <v>4</v>
@@ -2150,10 +2147,10 @@
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
       <c r="I45" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
@@ -2164,13 +2161,13 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>129</v>
       </c>
       <c r="E46" s="1">
         <v>4</v>
@@ -2179,10 +2176,10 @@
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
       <c r="I46" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
@@ -2193,13 +2190,13 @@
         <v>46</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E47" s="1">
         <v>4</v>
@@ -2218,13 +2215,13 @@
         <v>47</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E48" s="1">
         <v>3</v>
@@ -2243,13 +2240,13 @@
         <v>48</v>
       </c>
       <c r="B49" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D49" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>135</v>
       </c>
       <c r="E49" s="1">
         <v>2</v>
@@ -2268,13 +2265,13 @@
         <v>49</v>
       </c>
       <c r="B50" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D50" s="2" t="s">
         <v>136</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>138</v>
       </c>
       <c r="E50" s="1">
         <v>1</v>
@@ -2293,13 +2290,13 @@
         <v>50</v>
       </c>
       <c r="B51" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D51" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>141</v>
       </c>
       <c r="E51" s="1">
         <v>1</v>
@@ -2318,13 +2315,13 @@
         <v>51</v>
       </c>
       <c r="B52" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D52" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>144</v>
       </c>
       <c r="E52" s="1">
         <v>1</v>
@@ -2343,13 +2340,13 @@
         <v>52</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E53" s="1">
         <v>1</v>
@@ -2368,13 +2365,13 @@
         <v>53</v>
       </c>
       <c r="B54" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D54" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>149</v>
       </c>
       <c r="E54" s="1">
         <v>2</v>
@@ -2383,10 +2380,10 @@
       <c r="G54" s="1"/>
       <c r="H54" s="1"/>
       <c r="I54" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="K54" s="1"/>
       <c r="L54" s="1"/>
@@ -2397,13 +2394,13 @@
         <v>54</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E55" s="1">
         <v>1</v>
@@ -2412,10 +2409,10 @@
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
       <c r="I55" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="K55" s="1"/>
       <c r="L55" s="1"/>
@@ -2426,13 +2423,13 @@
         <v>55</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E56" s="1">
         <v>1</v>
@@ -2441,10 +2438,10 @@
       <c r="G56" s="1"/>
       <c r="H56" s="1"/>
       <c r="I56" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="K56" s="1"/>
       <c r="L56" s="1"/>

</xml_diff>